<commit_message>
Cost report: add t2.micro vs t3.micro, Linux vs Windows comparison
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/aws-detailed-cost-report.xlsx
+++ b/aws-detailed-cost-report.xlsx
@@ -5139,7 +5139,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -5879,11 +5879,226 @@
         </is>
       </c>
     </row>
+    <row r="35"/>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>E. Why t3.micro: t2.micro vs t3.micro, Linux vs Windows</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>Every stack runs Amazon Linux 2023 (AMI from the SSM parameter /aws/service/ami-amazon-linux-latest/al2023-ami-kernel-default-x86_64), so Linux prices apply. The operating system of the PC that runs Terraform (Windows here) has no effect on the AWS bill; only the instance's operating system does.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="42" customHeight="1">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Instance type / OS</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>vCPU / memory</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Per hour (USD)</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Per day (USD)</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>Per month (USD)</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>Note (hourly price is the blue input cell)</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Extra per month vs t3.micro Linux (USD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>t3.micro, Linux (used in every stack)</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>2 vCPU / 1 GiB</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>x86 (Intel)</t>
+        </is>
+      </c>
+      <c r="D39" s="43">
+        <f>D6</f>
+        <v>0.0104</v>
+      </c>
+      <c r="E39" s="43">
+        <f>D39*24</f>
+        <v>0.2496</v>
+      </c>
+      <c r="F39" s="43">
+        <f>D39*Rates!$B$4</f>
+        <v>7.592</v>
+      </c>
+      <c r="G39" s="15" t="inlineStr">
+        <is>
+          <t>Our choice. Linked to the t3.micro price in section A.</t>
+        </is>
+      </c>
+      <c r="H39" s="43">
+        <f>F39-$F$39</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>t2.micro, Linux</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>1 vCPU / 1 GiB</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>x86 (Intel)</t>
+        </is>
+      </c>
+      <c r="D40" s="40" t="n">
+        <v>0.0116</v>
+      </c>
+      <c r="E40" s="43">
+        <f>D40*24</f>
+        <v>0.2784</v>
+      </c>
+      <c r="F40" s="43">
+        <f>D40*Rates!$B$4</f>
+        <v>8.468</v>
+      </c>
+      <c r="G40" s="15" t="inlineStr">
+        <is>
+          <t>Older generation: about 10% dearer than t3.micro and half the vCPUs.</t>
+        </is>
+      </c>
+      <c r="H40" s="43">
+        <f>F40-$F$39</f>
+        <v>0.8760000000000003</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>t3.micro, Windows Server</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>2 vCPU / 1 GiB</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>x86 (Intel)</t>
+        </is>
+      </c>
+      <c r="D41" s="40" t="n">
+        <v>0.0196</v>
+      </c>
+      <c r="E41" s="43">
+        <f>D41*24</f>
+        <v>0.4704</v>
+      </c>
+      <c r="F41" s="43">
+        <f>D41*Rates!$B$4</f>
+        <v>14.308</v>
+      </c>
+      <c r="G41" s="15" t="inlineStr">
+        <is>
+          <t>Windows licence is billed per vCPU, so 2 vCPUs pay it twice.</t>
+        </is>
+      </c>
+      <c r="H41" s="43">
+        <f>F41-$F$39</f>
+        <v>6.716</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>t2.micro, Windows Server</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>1 vCPU / 1 GiB</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>x86 (Intel)</t>
+        </is>
+      </c>
+      <c r="D42" s="40" t="n">
+        <v>0.0162</v>
+      </c>
+      <c r="E42" s="43">
+        <f>D42*24</f>
+        <v>0.3888</v>
+      </c>
+      <c r="F42" s="43">
+        <f>D42*Rates!$B$4</f>
+        <v>11.825999999999999</v>
+      </c>
+      <c r="G42" s="15" t="inlineStr">
+        <is>
+          <t>Cheaper than t3.micro on Windows (1 vCPU licence), dearer than either on Linux.</t>
+        </is>
+      </c>
+      <c r="H42" s="43">
+        <f>F42-$F$39</f>
+        <v>4.233999999999999</v>
+      </c>
+    </row>
+    <row r="43" ht="45" customHeight="1">
+      <c r="A43" s="12" t="inlineStr">
+        <is>
+          <t>Why t3.micro: on Linux it is the cheapest x86 option ($0.0104/hr against $0.0116 for t2.micro) and has 2 vCPUs instead of 1. On Windows the order flips, because the Windows licence is charged per vCPU. Windows would also need a 30 GiB root volume ($2.40/month gp3, against $0.64 for the 8 GiB Linux root) and bigger snapshots and backups, so a Windows stack would cost roughly $14-16/month instead of $8-12.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="5">
     <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A43:H43"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A37:H37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Replace ec2-06 with a standalone EBS volume (no instance, no protection)
ec2-06 was the 1-vault AWS Backup stack; ec2-07 already covers that path.
It is now one encrypted 1 GiB gp3 volume, never attached, to test that an
unattached volume is found and scored on its own ($0.08/month).
Cost report and README updated: all 10 EC2 stacks now $96.95/month.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/aws-detailed-cost-report.xlsx
+++ b/aws-detailed-cost-report.xlsx
@@ -887,20 +887,20 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>ec2-06: Instance backup, 1 vault, no copy, no lock</t>
+          <t>ec2-06: Standalone 1 GiB gp3 volume, no instance, no protection</t>
         </is>
       </c>
       <c r="C11" s="35">
         <f>'Our stacks'!J15</f>
-        <v>0.016345205479452056</v>
+        <v>0.00010958904109589041</v>
       </c>
       <c r="D11" s="35">
         <f>'Our stacks'!K15</f>
-        <v>0.39228493150684934</v>
+        <v>0.00263013698630137</v>
       </c>
       <c r="E11" s="35">
         <f>'Our stacks'!L15</f>
-        <v>11.932</v>
+        <v>0.08</v>
       </c>
       <c r="F11" s="35">
         <f>'Our stacks'!M15</f>
@@ -1057,15 +1057,15 @@
       </c>
       <c r="C16" s="36">
         <f>'Our stacks'!J20</f>
-        <v>0.14904109589041098</v>
+        <v>0.1328054794520548</v>
       </c>
       <c r="D16" s="36">
         <f>'Our stacks'!K20</f>
-        <v>3.576986301369863</v>
+        <v>3.1873315068493153</v>
       </c>
       <c r="E16" s="36">
         <f>'Our stacks'!L20</f>
-        <v>108.8</v>
+        <v>96.948</v>
       </c>
       <c r="F16" s="36">
         <f>'Our stacks'!M20</f>
@@ -1975,7 +1975,7 @@
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>Public IPv4 (auto-assigned, ec2-01 to ec2-07, while running)</t>
+          <t>Public IPv4 (auto-assigned, ec2-01 to ec2-05, ec2-07, while running)</t>
         </is>
       </c>
       <c r="C49" s="37">
@@ -2309,7 +2309,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>A. EC2 folders (ec2/): every instance is left running</t>
+          <t>A. EC2 folders (ec2/): every instance is left running (ec2-06 has no instance)</t>
         </is>
       </c>
       <c r="B4" s="4" t="n"/>
@@ -2463,19 +2463,19 @@
       </c>
       <c r="B11" s="50" t="str">
         <f>'Our stacks'!B15</f>
-        <v>Instance backup, 1 vault, no copy, no lock</v>
+        <v>Standalone 1 GiB gp3 volume, no instance, no protection</v>
       </c>
       <c r="C11" s="51">
         <f>'Our stacks'!J15</f>
-        <v>0.016345205479452056</v>
+        <v>0.00010958904109589041</v>
       </c>
       <c r="D11" s="51">
         <f>'Our stacks'!O15</f>
-        <v>0.0009452054794520548</v>
+        <v>0.00010958904109589041</v>
       </c>
       <c r="E11" s="52">
         <f>'Our stacks'!L15</f>
-        <v>11.932</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="12">
@@ -2575,15 +2575,15 @@
       <c r="B16" s="53" t="n"/>
       <c r="C16" s="54">
         <f>SUM(C6:C15)</f>
-        <v>0.14904109589041098</v>
+        <v>0.1328054794520548</v>
       </c>
       <c r="D16" s="54">
         <f>SUM(D6:D15)</f>
-        <v>0.010041095890410958</v>
+        <v>0.009205479452054795</v>
       </c>
       <c r="E16" s="55">
         <f>SUM(E6:E15)</f>
-        <v>108.8</v>
+        <v>96.948</v>
       </c>
     </row>
     <row r="17"/>
@@ -3002,7 +3002,7 @@
     <row r="2" ht="39" customHeight="1">
       <c r="A2" s="12" t="inlineStr">
         <is>
-          <t>One row per folder in ec2/ and per AWS Backup folder in s3/. Quantities follow each main.tf; rates come from the Rates sheet. Per hour = compute + public IPv4 (while running) + EBS + snapshots + vault storage. One-time = the first cross-region copy, made by the first daily copy, or at apply in ec2-07 and ec2-09 (one on-demand backup job + one copy job). ec2-06, ec2-08 and ec2-backup-dr print the on-demand commands to run by hand. Every later daily copy sends only changed blocks.</t>
+          <t>One row per folder in ec2/ and per AWS Backup folder in s3/. Quantities follow each main.tf; rates come from the Rates sheet. Per hour = compute + public IPv4 (while running) + EBS + snapshots + vault storage. One-time = the first cross-region copy, made by the first daily copy, or at apply in ec2-07 and ec2-09 (one on-demand backup job + one copy job). ec2-08 and ec2-backup-dr print the on-demand commands to run by hand. Every later daily copy sends only changed blocks.</t>
         </is>
       </c>
     </row>
@@ -3530,28 +3530,27 @@
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>Instance backup, 1 vault, no copy, no lock</t>
+          <t>Standalone 1 GiB gp3 volume, no instance, no protection</t>
         </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>Running</t>
+          <t>None</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E15" s="20" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F15" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="G15" s="21">
-        <f>$C$4</f>
-        <v>1</v>
+      <c r="G15" s="21" t="n">
+        <v>0</v>
       </c>
       <c r="H15" s="21" t="n">
         <v>0</v>
@@ -3561,31 +3560,31 @@
       </c>
       <c r="J15" s="38">
         <f>IF(C15="Running",N15,O15)</f>
-        <v>0.016345205479452056</v>
+        <v>0.00010958904109589041</v>
       </c>
       <c r="K15" s="39">
         <f>J15*24</f>
-        <v>0.39228493150684934</v>
+        <v>0.00263013698630137</v>
       </c>
       <c r="L15" s="39">
         <f>J15*Rates!$B$4</f>
-        <v>11.932</v>
+        <v>0.08</v>
       </c>
       <c r="M15" s="39">
         <f>I15*Rates!$B$22</f>
         <v>0.0</v>
       </c>
       <c r="N15" s="39">
-        <f>'EC2 and EBS'!$D$6+IF(D15="Yes",Rates!$B$27,0)+O15</f>
-        <v>0.016345205479452056</v>
+        <f>O15</f>
+        <v>0.00010958904109589041</v>
       </c>
       <c r="O15" s="39">
         <f>(E15*Rates!$B$16+F15*Rates!$B$17+(G15+H15)*Rates!$B$20)/Rates!$B$4</f>
-        <v>0.0009452054794520548</v>
+        <v>0.00010958904109589041</v>
       </c>
       <c r="P15" s="15" t="inlineStr">
         <is>
-          <t>Daily 03:00 UTC, kept 1 day. On-demand backup: run the commands from terraform output (not at apply).</t>
+          <t>Unattached encrypted volume; nothing to stop, destroy to stop billing.</t>
         </is>
       </c>
     </row>
@@ -3881,15 +3880,15 @@
       <c r="I20" s="17" t="n"/>
       <c r="J20" s="38">
         <f>SUM(J10:J19)</f>
-        <v>0.14904109589041098</v>
+        <v>0.1328054794520548</v>
       </c>
       <c r="K20" s="38">
         <f>SUM(K10:K19)</f>
-        <v>3.576986301369863</v>
+        <v>3.1873315068493153</v>
       </c>
       <c r="L20" s="38">
         <f>SUM(L10:L19)</f>
-        <v>108.8</v>
+        <v>96.948</v>
       </c>
       <c r="M20" s="38">
         <f>SUM(M10:M19)</f>
@@ -4738,7 +4737,7 @@
       </c>
       <c r="E27" s="18" t="inlineStr">
         <is>
-          <t>ec2-01 to ec2-07 launch in default-VPC subnets, which auto-assign one: billed while the instance runs, released when it stops. ec2-08, ec2-09 and ec2-backup-dr set associate_public_ip_address = false, so they have none.</t>
+          <t>ec2-01 to ec2-05 and ec2-07 launch in default-VPC subnets, which auto-assign one: billed while the instance runs, released when it stops. ec2-08, ec2-09 and ec2-backup-dr set associate_public_ip_address = false, so they have none; ec2-06 has no instance.</t>
         </is>
       </c>
     </row>
@@ -5400,7 +5399,7 @@
       </c>
       <c r="G12" s="15" t="inlineStr">
         <is>
-          <t>ec2-01 to ec2-07 get one from the default VPC. Released (and no longer billed) when the instance stops. ec2-08, ec2-09 and ec2-backup-dr assign none.</t>
+          <t>ec2-01 to ec2-05 and ec2-07 get one from the default VPC. Released (and no longer billed) when the instance stops. ec2-08, ec2-09 and ec2-backup-dr assign none; ec2-06 has no instance.</t>
         </is>
       </c>
     </row>
@@ -5483,7 +5482,7 @@
       </c>
       <c r="G16" s="15" t="inlineStr">
         <is>
-          <t>The data volume in ec2-02 to ec2-05, ec2-09 and ec2-backup-dr.</t>
+          <t>The data volume in ec2-02 to ec2-05, ec2-09 and ec2-backup-dr, and the standalone volume in ec2-06.</t>
         </is>
       </c>
     </row>
@@ -5514,7 +5513,7 @@
       </c>
       <c r="G17" s="15" t="inlineStr">
         <is>
-          <t>The root volume in every EC2 stack.</t>
+          <t>The root volume in every EC2 stack except ec2-06, which has no instance.</t>
         </is>
       </c>
     </row>
@@ -6321,7 +6320,7 @@
       </c>
       <c r="G9" s="15" t="inlineStr">
         <is>
-          <t>Instance config + root volume snapshot, billed on used blocks. ec2-06, ec2-07, ec2-08.</t>
+          <t>Instance config + root volume snapshot, billed on used blocks. ec2-07, ec2-08.</t>
         </is>
       </c>
       <c r="H9" s="16" t="n"/>

</xml_diff>